<commit_message>
Completed Week 3 Assignment
</commit_message>
<xml_diff>
--- a/testfiles/Tests.xlsx
+++ b/testfiles/Tests.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10125"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xiesiyuan/Documents/FinTech-545/testfiles/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21F30B91-92DA-5447-9CA8-2C4AD0C2438A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65D3B3B6-B662-2343-A98A-C7212746CB83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="18980" yWindow="9000" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19380" yWindow="6200" windowWidth="18540" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -245,8 +245,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <strike/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -274,9 +282,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -583,61 +595,61 @@
       </c>
     </row>
     <row r="2" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A2">
+      <c r="A2" s="2">
         <v>1.1000000000000001</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D2" t="str">
+      <c r="D2" s="2" t="str">
         <f>"testout_"&amp;A2&amp;".csv"</f>
         <v>testout_1.1.csv</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A3">
+      <c r="A3" s="2">
         <v>1.2</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D3" t="str">
+      <c r="D3" s="2" t="str">
         <f t="shared" ref="D3:D40" si="0">"testout_"&amp;A3&amp;".csv"</f>
         <v>testout_1.2.csv</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A4">
+      <c r="A4" s="2">
         <v>1.3</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D4" t="str">
+      <c r="D4" s="2" t="str">
         <f t="shared" si="0"/>
         <v>testout_1.3.csv</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A5">
+      <c r="A5" s="2">
         <v>1.4</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D5" t="str">
+      <c r="D5" s="2" t="str">
         <f t="shared" si="0"/>
         <v>testout_1.4.csv</v>
       </c>
@@ -658,16 +670,16 @@
       </c>
     </row>
     <row r="7" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A7">
+      <c r="A7" s="2">
         <v>2.2000000000000002</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D7" t="str">
+      <c r="D7" s="2" t="str">
         <f t="shared" si="0"/>
         <v>testout_2.2.csv</v>
       </c>
@@ -688,76 +700,76 @@
       </c>
     </row>
     <row r="9" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A9">
+      <c r="A9" s="2">
         <v>3.1</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D9" t="str">
+      <c r="D9" s="2" t="str">
         <f t="shared" si="0"/>
         <v>testout_3.1.csv</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A10">
+      <c r="A10" s="2">
         <v>3.2</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D10" t="str">
+      <c r="D10" s="2" t="str">
         <f t="shared" si="0"/>
         <v>testout_3.2.csv</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A11">
+      <c r="A11" s="2">
         <v>3.3</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D11" t="str">
+      <c r="D11" s="2" t="str">
         <f t="shared" si="0"/>
         <v>testout_3.3.csv</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A12">
+      <c r="A12" s="2">
         <v>3.4</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D12" t="str">
+      <c r="D12" s="2" t="str">
         <f t="shared" si="0"/>
         <v>testout_3.4.csv</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A13">
+      <c r="A13" s="2">
         <v>4.0999999999999996</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B13" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D13" t="str">
+      <c r="D13" s="2" t="str">
         <f t="shared" si="0"/>
         <v>testout_4.1.csv</v>
       </c>
@@ -838,76 +850,76 @@
       </c>
     </row>
     <row r="19" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A19">
+      <c r="A19" s="2">
         <v>6.1</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="B19" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C19" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D19" t="str">
+      <c r="D19" s="2" t="str">
         <f t="shared" si="0"/>
         <v>testout_6.1.csv</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A20">
+      <c r="A20" s="2">
         <v>6.2</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B20" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C20" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D20" t="str">
+      <c r="D20" s="2" t="str">
         <f t="shared" si="0"/>
         <v>testout_6.2.csv</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A21">
+      <c r="A21" s="2">
         <v>7.1</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="B21" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C21" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="D21" t="str">
+      <c r="D21" s="2" t="str">
         <f t="shared" si="0"/>
         <v>testout_7.1.csv</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A22">
+      <c r="A22" s="2">
         <v>7.2</v>
       </c>
-      <c r="B22" s="1" t="s">
+      <c r="B22" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C22" t="s">
+      <c r="C22" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="D22" t="str">
+      <c r="D22" s="2" t="str">
         <f t="shared" si="0"/>
         <v>testout_7.2.csv</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A23">
+      <c r="A23" s="2">
         <v>7.3</v>
       </c>
-      <c r="B23" s="1" t="s">
+      <c r="B23" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="C23" t="s">
+      <c r="C23" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="D23" t="str">
+      <c r="D23" s="2" t="str">
         <f t="shared" si="0"/>
         <v>testout_7.3.csv</v>
       </c>

</xml_diff>

<commit_message>
Completed Week 4 Assignment
</commit_message>
<xml_diff>
--- a/testfiles/Tests.xlsx
+++ b/testfiles/Tests.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10125"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10208"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xiesiyuan/Documents/FinTech-545/testfiles/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65D3B3B6-B662-2343-A98A-C7212746CB83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B92B8983-8682-5241-8C60-19259B91D5EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19380" yWindow="6200" windowWidth="18540" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="400" yWindow="7260" windowWidth="18540" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -655,16 +655,16 @@
       </c>
     </row>
     <row r="6" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A6">
+      <c r="A6" s="2">
         <v>2.1</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D6" t="str">
+      <c r="D6" s="2" t="str">
         <f t="shared" si="0"/>
         <v>testout_2.1.csv</v>
       </c>
@@ -685,16 +685,16 @@
       </c>
     </row>
     <row r="8" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A8">
+      <c r="A8" s="2">
         <v>2.2999999999999998</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D8" t="str">
+      <c r="D8" s="2" t="str">
         <f t="shared" si="0"/>
         <v>testout_2.3.csv</v>
       </c>
@@ -775,61 +775,61 @@
       </c>
     </row>
     <row r="14" spans="1:4" ht="32" x14ac:dyDescent="0.2">
-      <c r="A14">
+      <c r="A14" s="2">
         <v>5.0999999999999996</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="D14" t="str">
+      <c r="D14" s="2" t="str">
         <f t="shared" si="0"/>
         <v>testout_5.1.csv</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="32" x14ac:dyDescent="0.2">
-      <c r="A15">
+      <c r="A15" s="2">
         <v>5.2</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B15" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D15" t="str">
+      <c r="D15" s="2" t="str">
         <f t="shared" si="0"/>
         <v>testout_5.2.csv</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="32" x14ac:dyDescent="0.2">
-      <c r="A16">
+      <c r="A16" s="2">
         <v>5.3</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B16" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C16" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="D16" t="str">
+      <c r="D16" s="2" t="str">
         <f t="shared" si="0"/>
         <v>testout_5.3.csv</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="32" x14ac:dyDescent="0.2">
-      <c r="A17">
+      <c r="A17" s="2">
         <v>5.4</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B17" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C17" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="D17" t="str">
+      <c r="D17" s="2" t="str">
         <f t="shared" si="0"/>
         <v>testout_5.4.csv</v>
       </c>
@@ -940,31 +940,31 @@
       </c>
     </row>
     <row r="25" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A25">
+      <c r="A25" s="2">
         <v>8.1</v>
       </c>
-      <c r="B25" s="1" t="s">
+      <c r="B25" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="C25" t="s">
+      <c r="C25" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="D25" t="str">
+      <c r="D25" s="2" t="str">
         <f t="shared" si="0"/>
         <v>testout_8.1.csv</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A26">
+      <c r="A26" s="2">
         <v>8.1999999999999993</v>
       </c>
-      <c r="B26" s="1" t="s">
+      <c r="B26" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C26" t="s">
+      <c r="C26" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="D26" t="str">
+      <c r="D26" s="2" t="str">
         <f t="shared" si="0"/>
         <v>testout_8.2.csv</v>
       </c>

</xml_diff>